<commit_message>
One figure comparing many GHG pricing schemes
</commit_message>
<xml_diff>
--- a/config-aggregation/aggregations_git.xlsx
+++ b/config-aggregation/aggregations_git.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ladi\ZHAWonTresorit\Projects\Caritas\PSI-CCL_HABE\CCL-results_fromGithub\config-aggregation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20D99142-6342-44CC-AF3F-EE326563C076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34EC741E-1A12-41A3-9D0C-DE85EBF1D162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3digit" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="check_gwp_list" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">cprice_versions!$A$3:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">cprice_versions!$A$5:$B$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2035" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2046" uniqueCount="292">
   <si>
     <t>gwp42</t>
   </si>
@@ -1015,6 +1015,9 @@
   </si>
   <si>
     <t>Sports, recreation, holidays</t>
+  </si>
+  <si>
+    <t>All transport</t>
   </si>
 </sst>
 </file>
@@ -6923,7 +6926,7 @@
         <v>Equal</v>
       </c>
       <c r="GL5" t="str">
-        <f t="shared" ref="GL5:IW5" si="3">IF(GL3&lt;&gt;GL1,"Different!",IF(GL2&lt;&gt;GL1,"Different!",IF(GL4&lt;&gt;GL1,"Different!","Equal")))</f>
+        <f t="shared" ref="GL5:GV5" si="3">IF(GL3&lt;&gt;GL1,"Different!",IF(GL2&lt;&gt;GL1,"Different!",IF(GL4&lt;&gt;GL1,"Different!","Equal")))</f>
         <v>Equal</v>
       </c>
       <c r="GM5" t="str">
@@ -9718,7 +9721,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D07E399-6037-41CA-8A56-1674D00BF41C}">
-  <dimension ref="A1:GZ10"/>
+  <dimension ref="A1:GZ11"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="37.140625" style="1" bestFit="1" customWidth="1"/>
@@ -10960,225 +10963,261 @@
     </row>
     <row r="3" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CO3" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CP3" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CQ3" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="DI3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="DJ3" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ3" s="2"/>
     </row>
     <row r="4" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="CS4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CT4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CU4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CV4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CW4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CX4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CY4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="CZ4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="DA4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="DB4" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="DC4" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="EG4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EH4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EI4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EJ4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EK4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EL4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GN4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GO4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GS4" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GT4" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ4" s="2"/>
     </row>
     <row r="5" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="DI5" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="DJ5" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="CO5" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CP5" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CQ5" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ5" s="2"/>
     </row>
     <row r="6" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="EG6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EH6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EI6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EK6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EL6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GN6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GO6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GS6" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GT6" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="CS6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CT6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CU6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CV6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CW6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CX6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CY6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="CZ6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="DA6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="DB6" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="DC6" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ6" s="2"/>
     </row>
     <row r="7" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="EJ7" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="EG7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EH7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EI7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EK7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EL7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GN7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GO7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GS7" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GT7" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ7" s="2"/>
     </row>
     <row r="8" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="CR8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EU8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EV8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EW8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EX8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EY8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="EZ8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FA8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FB8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FC8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FD8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FE8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FF8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FG8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FH8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FI8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FJ8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FK8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FL8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FM8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FN8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FO8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FP8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FQ8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FR8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FS8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FT8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FU8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FV8" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="FW8" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="EJ8" s="1" t="s">
         <v>202</v>
       </c>
       <c r="GZ8" s="2"/>
     </row>
     <row r="9" spans="1:208" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="CR9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EU9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EV9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EW9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EX9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EY9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="EZ9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FA9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FB9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FC9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FD9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FE9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FF9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FG9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FH9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FI9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FJ9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FK9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FL9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FM9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FN9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FO9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FP9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FQ9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FR9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FS9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FT9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FU9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FV9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="FW9" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GZ9" s="2"/>
+    </row>
+    <row r="10" spans="1:208" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="GF9" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GG9" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GH9" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="GZ9" s="2"/>
-    </row>
-    <row r="10" spans="1:208" x14ac:dyDescent="0.2">
+      <c r="GF10" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GG10" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="GH10" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="GZ10" s="2"/>
+    </row>
+    <row r="11" spans="1:208" x14ac:dyDescent="0.2">
+      <c r="GZ11" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>